<commit_message>
docs: koreksi asumsi PPN di proyeksi finansial (harga di Play tanpa PPN) dan teks keterangan PPN
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/PROYEKSI-FINANSIAL.xlsx
+++ b/docs/PROYEKSI-FINANSIAL.xlsx
@@ -559,7 +559,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Disusun 2026-10-05. PERKIRAAN dari asumsi, bukan ramalan dan bukan nasihat pajak.</t>
+          <t>Disusun 2026-10-05; asumsi PPN dikoreksi 2026-10-09 setelah pesanan nyata pertama. PERKIRAAN dari asumsi, bukan ramalan dan bukan nasihat pajak.</t>
         </is>
       </c>
     </row>
@@ -699,7 +699,7 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Harga Play di Indonesia diasumsikan sudah termasuk PPN (efektif 11%), dipungut dan disetor Google. VERIFIKASI di Play Console.</t>
+          <t>Harga di Play (Rp7.500, Rp12.500, dst.) adalah harga JUAL tanpa PPN. PPN 11% ditambahkan di atas harga dan dipungut/disetor Google, jadi pelanggan Ultimate bulanan membayar Rp13.875. Biaya Google 15% dihitung dari harga jual. TERVERIFIKASI dari pesanan nyata 2026-10-09.</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
-          <t>Harga langganan (Rp, harga yang tampil di Play)</t>
+          <t>Harga langganan (Rp, harga jual di Play, BELUM termasuk PPN)</t>
         </is>
       </c>
       <c r="B3" s="10" t="n"/>
@@ -946,22 +946,22 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>12% dengan DPP nilai lain 11/12 = efektif 11%. Konfirmasi ke konsultan pajak.</t>
+          <t>11% (pajak Rp1.375 atas harga jual Rp12.500 di pesanan nyata). Konfirmasi status ke konsultan pajak.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>Harga Play sudah termasuk PPN? (1 = ya, 0 = belum)</t>
+          <t>Harga Play sudah termasuk PPN? (1 = ya, 0 = belum; PPN ditambahkan di atas harga)</t>
         </is>
       </c>
       <c r="B12" s="15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>ASUMSI: ya. VERIFIKASI di Play Console &gt; Monetisasi &gt; Produk. Jika 0, net naik ~10%.</t>
+          <t>TERVERIFIKASI 2026-10-09 dari pesanan Play GPA.3304-9982-3764-47106: harga jual Rp12.500 + pajak Rp1.375 = total Rp13.875; estimasi pendapatan USD 0,59 = Rp12.500 x 85% / Rp17.930. Pelanggan membayar PPN di atas harga; Google memungut dan menyetornya.</t>
         </is>
       </c>
     </row>
@@ -1361,7 +1361,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -1381,7 +1381,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Dari harga yang dibayar sampai net yang Anda terima. Semua dihitung dari sheet Asumsi.</t>
+          <t>Dari harga jual sampai net yang Anda terima. PPN dibayar pelanggan di atas harga (baris informasi di bawah). Semua dihitung dari sheet Asumsi.</t>
         </is>
       </c>
     </row>
@@ -1406,7 +1406,7 @@
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Harga efektif per bulan (campuran bulanan/tahunan)</t>
+          <t>Harga jual efektif per bulan (campuran bulanan/tahunan, tanpa PPN)</t>
         </is>
       </c>
       <c r="B4" s="21">
@@ -1425,44 +1425,44 @@
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
         <is>
-          <t>PPN termasuk dalam harga (dipungut Google)</t>
+          <t>PPN yang dipotong dari harga (0 bila PPN di atas harga)</t>
         </is>
       </c>
       <c r="B5" s="21">
         <f>IF(Asumsi!$B$12=1,B4-B4/(1+Asumsi!$B$11),0)</f>
-        <v>693.6936936936945</v>
+        <v>0</v>
       </c>
       <c r="C5" s="21">
         <f>IF(Asumsi!$B$12=1,C4-C4/(1+Asumsi!$B$11),0)</f>
-        <v>1156.1561561561575</v>
+        <v>0</v>
       </c>
       <c r="D5" s="21">
         <f>IF(Asumsi!$B$12=1,D4-D4/(1+Asumsi!$B$11),0)</f>
-        <v>1156.1561561561575</v>
+        <v>0</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Bernilai 0 bila 'Harga Play sudah termasuk PPN' = 0.</t>
+          <t>Bernilai 0 karena 'Harga Play sudah termasuk PPN' = 0: PPN ditambahkan di atas harga, bukan dipotong dari pendapatan Anda.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>Dasar sebelum biaya Google</t>
+          <t>Dasar biaya Google (harga jual)</t>
         </is>
       </c>
       <c r="B6" s="21">
         <f>B4-B5</f>
-        <v>6306.3063063063055</v>
+        <v>7000.0</v>
       </c>
       <c r="C6" s="21">
         <f>C4-C5</f>
-        <v>10510.51051051051</v>
+        <v>11666.666666666668</v>
       </c>
       <c r="D6" s="21">
         <f>D4-D5</f>
-        <v>10510.51051051051</v>
+        <v>11666.666666666668</v>
       </c>
     </row>
     <row r="7">
@@ -1473,15 +1473,15 @@
       </c>
       <c r="B7" s="21">
         <f>B6*Asumsi!$B$13</f>
-        <v>945.9459459459458</v>
+        <v>1050.0</v>
       </c>
       <c r="C7" s="21">
         <f>C6*Asumsi!$B$13</f>
-        <v>1576.5765765765766</v>
+        <v>1750.0000000000002</v>
       </c>
       <c r="D7" s="21">
         <f>D6*Asumsi!$B$13</f>
-        <v>1576.5765765765766</v>
+        <v>1750.0000000000002</v>
       </c>
     </row>
     <row r="8">
@@ -1515,15 +1515,15 @@
       </c>
       <c r="B9" s="23">
         <f>B6-B7-B8</f>
-        <v>5360.36036036036</v>
+        <v>5950.0</v>
       </c>
       <c r="C9" s="23">
         <f>C6-C7-C8</f>
-        <v>8675.933933933933</v>
+        <v>9658.666666666668</v>
       </c>
       <c r="D9" s="23">
         <f>D6-D7-D8</f>
-        <v>6653.933933933933</v>
+        <v>7636.666666666668</v>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
@@ -1534,39 +1534,39 @@
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>Net sebagai persen dari harga</t>
+          <t>Net sebagai persen dari harga jual</t>
         </is>
       </c>
       <c r="B10" s="24">
         <f>IF(B4=0,0,B9/B4)</f>
-        <v>0.7657657657657657</v>
+        <v>0.85</v>
       </c>
       <c r="C10" s="24">
         <f>IF(C4=0,0,C9/C4)</f>
-        <v>0.7436514800514799</v>
+        <v>0.8278857142857143</v>
       </c>
       <c r="D10" s="24">
         <f>IF(D4=0,0,D9/D4)</f>
-        <v>0.5703371943371942</v>
+        <v>0.6545714285714286</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
         <is>
-          <t>PPh final (skema PT/CV, per pelanggan)</t>
+          <t>PPh final (skema PT/CV, per pelanggan, dari harga jual)</t>
         </is>
       </c>
       <c r="B11" s="21">
         <f>B6*Asumsi!$B$14</f>
-        <v>31.531531531531527</v>
+        <v>35.0</v>
       </c>
       <c r="C11" s="21">
         <f>C6*Asumsi!$B$14</f>
-        <v>52.552552552552555</v>
+        <v>58.33333333333334</v>
       </c>
       <c r="D11" s="21">
         <f>D6*Asumsi!$B$14</f>
-        <v>52.552552552552555</v>
+        <v>58.33333333333334</v>
       </c>
     </row>
     <row r="12">
@@ -1577,15 +1577,77 @@
       </c>
       <c r="B12" s="23">
         <f>B9-B11</f>
-        <v>5328.828828828828</v>
+        <v>5915.0</v>
       </c>
       <c r="C12" s="23">
         <f>C9-C11</f>
-        <v>8623.381381381381</v>
+        <v>9600.333333333334</v>
       </c>
       <c r="D12" s="23">
         <f>D9-D11</f>
-        <v>6601.38138138138</v>
+        <v>7578.333333333335</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>Informasi: PPN yang ditambahkan Google di atas harga (dibayar pelanggan)</t>
+        </is>
+      </c>
+      <c r="B14" s="21">
+        <f>IF(Asumsi!$B$12=1,0,B4*Asumsi!$B$11)</f>
+        <v>770.0</v>
+      </c>
+      <c r="C14" s="21">
+        <f>IF(Asumsi!$B$12=1,0,C4*Asumsi!$B$11)</f>
+        <v>1283.3333333333335</v>
+      </c>
+      <c r="D14" s="21">
+        <f>IF(Asumsi!$B$12=1,0,D4*Asumsi!$B$11)</f>
+        <v>1283.3333333333335</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Bukan beban atau pendapatan Anda: Google yang memungut dan menyetor PPN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>Informasi: total yang dibayar pelanggan per bulan (harga + PPN)</t>
+        </is>
+      </c>
+      <c r="B15" s="21">
+        <f>B4+B14</f>
+        <v>7770.0</v>
+      </c>
+      <c r="C15" s="21">
+        <f>C4+C14</f>
+        <v>12950.000000000002</v>
+      </c>
+      <c r="D15" s="21">
+        <f>D4+D14</f>
+        <v>12950.000000000002</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>Informasi: net sebagai persen dari total yang dibayar pelanggan</t>
+        </is>
+      </c>
+      <c r="B16" s="24">
+        <f>IF(B15=0,0,B9/B15)</f>
+        <v>0.7657657657657657</v>
+      </c>
+      <c r="C16" s="24">
+        <f>IF(C15=0,0,C9/C15)</f>
+        <v>0.7458429858429858</v>
+      </c>
+      <c r="D16" s="24">
+        <f>IF(D15=0,0,D9/D15)</f>
+        <v>0.5897039897039897</v>
       </c>
     </row>
   </sheetData>
@@ -1599,7 +1661,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -1746,7 +1808,7 @@
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>Uang masuk dari pelanggan per bulan (bruto)</t>
+          <t>Uang masuk dari pelanggan per bulan (harga jual, tanpa PPN)</t>
         </is>
       </c>
       <c r="B10" s="21">
@@ -1765,39 +1827,39 @@
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
         <is>
-          <t>PPN (dipungut Google)</t>
+          <t>PPN yang dipotong dari harga (0 bila PPN di atas harga)</t>
         </is>
       </c>
       <c r="B11" s="21">
         <f>B8*Per_Pelanggan!$B$5+B7*Per_Pelanggan!$C$5</f>
-        <v>11792.792792792807</v>
+        <v>0.0</v>
       </c>
       <c r="C11" s="21">
         <f>C8*Per_Pelanggan!$B$5+C7*Per_Pelanggan!$C$5</f>
-        <v>101048.04804804816</v>
+        <v>0.0</v>
       </c>
       <c r="D11" s="21">
         <f>D8*Per_Pelanggan!$B$5+D7*Per_Pelanggan!$C$5</f>
-        <v>499459.45945946005</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>Dasar sebelum biaya Google</t>
+          <t>Dasar biaya Google (harga jual)</t>
         </is>
       </c>
       <c r="B12" s="21">
         <f>B10-B11</f>
-        <v>107207.20720720719</v>
+        <v>119000.0</v>
       </c>
       <c r="C12" s="21">
         <f>C10-C11</f>
-        <v>918618.6186186186</v>
+        <v>1019666.6666666667</v>
       </c>
       <c r="D12" s="21">
         <f>D10-D11</f>
-        <v>4540540.54054054</v>
+        <v>5040000.0</v>
       </c>
     </row>
     <row r="13">
@@ -1808,15 +1870,15 @@
       </c>
       <c r="B13" s="21">
         <f>B12*Asumsi!$B$13</f>
-        <v>16081.081081081078</v>
+        <v>17850.0</v>
       </c>
       <c r="C13" s="21">
         <f>C12*Asumsi!$B$13</f>
-        <v>137792.79279279278</v>
+        <v>152950.0</v>
       </c>
       <c r="D13" s="21">
         <f>D12*Asumsi!$B$13</f>
-        <v>681081.081081081</v>
+        <v>756000.0</v>
       </c>
     </row>
     <row r="14">
@@ -1884,15 +1946,15 @@
       </c>
       <c r="B17" s="23">
         <f>B12-B13-B14-B15-B16</f>
-        <v>90352.12612612611</v>
+        <v>100376.0</v>
       </c>
       <c r="C17" s="23">
         <f>C12-C13-C14-C15-C16</f>
-        <v>772827.8258258258</v>
+        <v>858718.6666666667</v>
       </c>
       <c r="D17" s="23">
         <f>D12-D13-D14-D15-D16</f>
-        <v>3813019.4594594585</v>
+        <v>4237560.0</v>
       </c>
     </row>
     <row r="18">
@@ -1903,15 +1965,15 @@
       </c>
       <c r="B18" s="21">
         <f>IF(Asumsi!$B$15=1,MAX(0,B12*12-Asumsi!$B$16)*Asumsi!$B$14/12,B12*Asumsi!$B$14)</f>
-        <v>536.036036036036</v>
+        <v>595.0</v>
       </c>
       <c r="C18" s="21">
         <f>IF(Asumsi!$B$15=1,MAX(0,C12*12-Asumsi!$B$16)*Asumsi!$B$14/12,C12*Asumsi!$B$14)</f>
-        <v>4593.093093093093</v>
+        <v>5098.333333333334</v>
       </c>
       <c r="D18" s="21">
         <f>IF(Asumsi!$B$15=1,MAX(0,D12*12-Asumsi!$B$16)*Asumsi!$B$14/12,D12*Asumsi!$B$14)</f>
-        <v>22702.7027027027</v>
+        <v>25200.0</v>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
@@ -1927,15 +1989,15 @@
       </c>
       <c r="B19" s="23">
         <f>B17-B18</f>
-        <v>89816.09009009007</v>
+        <v>99781.0</v>
       </c>
       <c r="C19" s="23">
         <f>C17-C18</f>
-        <v>768234.7327327327</v>
+        <v>853620.3333333334</v>
       </c>
       <c r="D19" s="23">
         <f>D17-D18</f>
-        <v>3790316.756756756</v>
+        <v>4212360.0</v>
       </c>
     </row>
     <row r="20">
@@ -1946,15 +2008,15 @@
       </c>
       <c r="B20" s="23">
         <f>B19*12</f>
-        <v>1077793.081081081</v>
+        <v>1197372.0</v>
       </c>
       <c r="C20" s="23">
         <f>C19*12</f>
-        <v>9218816.792792792</v>
+        <v>10243444.0</v>
       </c>
       <c r="D20" s="23">
         <f>D19*12</f>
-        <v>45483801.08108107</v>
+        <v>50548320.0</v>
       </c>
     </row>
     <row r="21">
@@ -1965,15 +2027,15 @@
       </c>
       <c r="B21" s="21">
         <f>B20*Asumsi!B41</f>
-        <v>538896.5405405405</v>
+        <v>598686.0</v>
       </c>
       <c r="C21" s="21">
         <f>C20*Asumsi!C41</f>
-        <v>4609408.396396396</v>
+        <v>5121722.0</v>
       </c>
       <c r="D21" s="21">
         <f>D20*Asumsi!D41</f>
-        <v>22741900.540540535</v>
+        <v>25274160.0</v>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
@@ -1984,20 +2046,20 @@
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
-          <t>Net bersih sebagai persen dari uang masuk</t>
+          <t>Net bersih sebagai persen dari harga jual</t>
         </is>
       </c>
       <c r="B22" s="24">
         <f>IF(B10=0,0,B19/B10)</f>
-        <v>0.7547570595805888</v>
+        <v>0.8384957983193277</v>
       </c>
       <c r="C22" s="24">
         <f>IF(C10=0,0,C19/C10)</f>
-        <v>0.7534175214770179</v>
+        <v>0.8371562602157567</v>
       </c>
       <c r="D22" s="24">
         <f>IF(D10=0,0,D19/D10)</f>
-        <v>0.7520469755469754</v>
+        <v>0.8357857142857142</v>
       </c>
     </row>
     <row r="23">
@@ -2034,15 +2096,15 @@
       </c>
       <c r="B25" s="21">
         <f>B12-B13-B24-B15-B16</f>
-        <v>84286.12612612611</v>
+        <v>94310.0</v>
       </c>
       <c r="C25" s="21">
         <f>C12-C13-C24-C15-C16</f>
-        <v>710145.8258258258</v>
+        <v>796036.6666666667</v>
       </c>
       <c r="D25" s="21">
         <f>D12-D13-D24-D15-D16</f>
-        <v>3449059.4594594585</v>
+        <v>3873600.0</v>
       </c>
     </row>
     <row r="26">
@@ -2122,15 +2184,58 @@
       </c>
       <c r="B30" s="21">
         <f>B19+B29</f>
-        <v>619647.5900900901</v>
+        <v>629612.5</v>
       </c>
       <c r="C30" s="21">
         <f>C19+C29</f>
-        <v>3390497.232732733</v>
+        <v>3475882.8333333335</v>
       </c>
       <c r="D30" s="21">
         <f>D19+D29</f>
-        <v>14225576.756756756</v>
+        <v>14647620.0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="11" t="inlineStr">
+        <is>
+          <t>Informasi: PPN yang ditambahkan Google di atas harga per bulan</t>
+        </is>
+      </c>
+      <c r="B32" s="21">
+        <f>IF(Asumsi!$B$12=1,0,B10*Asumsi!$B$11)</f>
+        <v>13090.0</v>
+      </c>
+      <c r="C32" s="21">
+        <f>IF(Asumsi!$B$12=1,0,C10*Asumsi!$B$11)</f>
+        <v>112163.33333333334</v>
+      </c>
+      <c r="D32" s="21">
+        <f>IF(Asumsi!$B$12=1,0,D10*Asumsi!$B$11)</f>
+        <v>554400.0</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Bukan beban Anda; dipungut dan disetor Google.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="11" t="inlineStr">
+        <is>
+          <t>Informasi: total yang dibayar semua pelanggan per bulan (harga + PPN)</t>
+        </is>
+      </c>
+      <c r="B33" s="21">
+        <f>B10+B32</f>
+        <v>132090.0</v>
+      </c>
+      <c r="C33" s="21">
+        <f>C10+C32</f>
+        <v>1131830.0</v>
+      </c>
+      <c r="D33" s="21">
+        <f>D10+D32</f>
+        <v>5594400.0</v>
       </c>
     </row>
   </sheetData>
@@ -2213,23 +2318,23 @@
       </c>
       <c r="B6" s="21">
         <f>$A6*B$5*((1-$B$3)*Per_Pelanggan!$B$9+$B$3*Per_Pelanggan!$C$9)*12-Asumsi!$B$34*12</f>
-        <v>371355.2252252252</v>
+        <v>412630.0</v>
       </c>
       <c r="C6" s="21">
         <f>$A6*C$5*((1-$B$3)*Per_Pelanggan!$B$9+$B$3*Per_Pelanggan!$C$9)*12-Asumsi!$B$34*12</f>
-        <v>742710.4504504504</v>
+        <v>825260.0</v>
       </c>
       <c r="D6" s="21">
         <f>$A6*D$5*((1-$B$3)*Per_Pelanggan!$B$9+$B$3*Per_Pelanggan!$C$9)*12-Asumsi!$B$34*12</f>
-        <v>1114065.6756756757</v>
+        <v>1237890.0</v>
       </c>
       <c r="E6" s="21">
         <f>$A6*E$5*((1-$B$3)*Per_Pelanggan!$B$9+$B$3*Per_Pelanggan!$C$9)*12-Asumsi!$B$34*12</f>
-        <v>1485420.9009009008</v>
+        <v>1650520.0</v>
       </c>
       <c r="F6" s="21">
         <f>$A6*F$5*((1-$B$3)*Per_Pelanggan!$B$9+$B$3*Per_Pelanggan!$C$9)*12-Asumsi!$B$34*12</f>
-        <v>1856776.1261261262</v>
+        <v>2063150.0000000002</v>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
@@ -2243,23 +2348,23 @@
       </c>
       <c r="B7" s="21">
         <f>$A7*B$5*((1-$B$3)*Per_Pelanggan!$B$9+$B$3*Per_Pelanggan!$C$9)*12-Asumsi!$B$34*12</f>
-        <v>742710.4504504504</v>
+        <v>825260.0</v>
       </c>
       <c r="C7" s="21">
         <f>$A7*C$5*((1-$B$3)*Per_Pelanggan!$B$9+$B$3*Per_Pelanggan!$C$9)*12-Asumsi!$B$34*12</f>
-        <v>1485420.9009009008</v>
+        <v>1650520.0</v>
       </c>
       <c r="D7" s="21">
         <f>$A7*D$5*((1-$B$3)*Per_Pelanggan!$B$9+$B$3*Per_Pelanggan!$C$9)*12-Asumsi!$B$34*12</f>
-        <v>2228131.3513513515</v>
+        <v>2475780.0</v>
       </c>
       <c r="E7" s="21">
         <f>$A7*E$5*((1-$B$3)*Per_Pelanggan!$B$9+$B$3*Per_Pelanggan!$C$9)*12-Asumsi!$B$34*12</f>
-        <v>2970841.8018018017</v>
+        <v>3301040.0</v>
       </c>
       <c r="F7" s="21">
         <f>$A7*F$5*((1-$B$3)*Per_Pelanggan!$B$9+$B$3*Per_Pelanggan!$C$9)*12-Asumsi!$B$34*12</f>
-        <v>3713552.2522522523</v>
+        <v>4126300.0000000005</v>
       </c>
     </row>
     <row r="8">
@@ -2268,23 +2373,23 @@
       </c>
       <c r="B8" s="21">
         <f>$A8*B$5*((1-$B$3)*Per_Pelanggan!$B$9+$B$3*Per_Pelanggan!$C$9)*12-Asumsi!$B$34*12</f>
-        <v>1856776.1261261262</v>
+        <v>2063150.0000000002</v>
       </c>
       <c r="C8" s="21">
         <f>$A8*C$5*((1-$B$3)*Per_Pelanggan!$B$9+$B$3*Per_Pelanggan!$C$9)*12-Asumsi!$B$34*12</f>
-        <v>3713552.2522522523</v>
+        <v>4126300.0000000005</v>
       </c>
       <c r="D8" s="21">
         <f>$A8*D$5*((1-$B$3)*Per_Pelanggan!$B$9+$B$3*Per_Pelanggan!$C$9)*12-Asumsi!$B$34*12</f>
-        <v>5570328.378378378</v>
+        <v>6189450.0</v>
       </c>
       <c r="E8" s="21">
         <f>$A8*E$5*((1-$B$3)*Per_Pelanggan!$B$9+$B$3*Per_Pelanggan!$C$9)*12-Asumsi!$B$34*12</f>
-        <v>7427104.504504505</v>
+        <v>8252600.000000001</v>
       </c>
       <c r="F8" s="21">
         <f>$A8*F$5*((1-$B$3)*Per_Pelanggan!$B$9+$B$3*Per_Pelanggan!$C$9)*12-Asumsi!$B$34*12</f>
-        <v>9283880.630630631</v>
+        <v>10315750.0</v>
       </c>
     </row>
     <row r="9">
@@ -2293,23 +2398,23 @@
       </c>
       <c r="B9" s="21">
         <f>$A9*B$5*((1-$B$3)*Per_Pelanggan!$B$9+$B$3*Per_Pelanggan!$C$9)*12-Asumsi!$B$34*12</f>
-        <v>3713552.2522522523</v>
+        <v>4126300.0000000005</v>
       </c>
       <c r="C9" s="21">
         <f>$A9*C$5*((1-$B$3)*Per_Pelanggan!$B$9+$B$3*Per_Pelanggan!$C$9)*12-Asumsi!$B$34*12</f>
-        <v>7427104.504504505</v>
+        <v>8252600.000000001</v>
       </c>
       <c r="D9" s="21">
         <f>$A9*D$5*((1-$B$3)*Per_Pelanggan!$B$9+$B$3*Per_Pelanggan!$C$9)*12-Asumsi!$B$34*12</f>
-        <v>11140656.756756756</v>
+        <v>12378900.0</v>
       </c>
       <c r="E9" s="21">
         <f>$A9*E$5*((1-$B$3)*Per_Pelanggan!$B$9+$B$3*Per_Pelanggan!$C$9)*12-Asumsi!$B$34*12</f>
-        <v>14854209.00900901</v>
+        <v>16505200.000000002</v>
       </c>
       <c r="F9" s="21">
         <f>$A9*F$5*((1-$B$3)*Per_Pelanggan!$B$9+$B$3*Per_Pelanggan!$C$9)*12-Asumsi!$B$34*12</f>
-        <v>18567761.261261262</v>
+        <v>20631500.0</v>
       </c>
     </row>
     <row r="10">
@@ -2318,23 +2423,23 @@
       </c>
       <c r="B10" s="21">
         <f>$A10*B$5*((1-$B$3)*Per_Pelanggan!$B$9+$B$3*Per_Pelanggan!$C$9)*12-Asumsi!$B$34*12</f>
-        <v>7427104.504504505</v>
+        <v>8252600.000000001</v>
       </c>
       <c r="C10" s="21">
         <f>$A10*C$5*((1-$B$3)*Per_Pelanggan!$B$9+$B$3*Per_Pelanggan!$C$9)*12-Asumsi!$B$34*12</f>
-        <v>14854209.00900901</v>
+        <v>16505200.000000002</v>
       </c>
       <c r="D10" s="21">
         <f>$A10*D$5*((1-$B$3)*Per_Pelanggan!$B$9+$B$3*Per_Pelanggan!$C$9)*12-Asumsi!$B$34*12</f>
-        <v>22281313.513513513</v>
+        <v>24757800.0</v>
       </c>
       <c r="E10" s="21">
         <f>$A10*E$5*((1-$B$3)*Per_Pelanggan!$B$9+$B$3*Per_Pelanggan!$C$9)*12-Asumsi!$B$34*12</f>
-        <v>29708418.01801802</v>
+        <v>33010400.000000004</v>
       </c>
       <c r="F10" s="21">
         <f>$A10*F$5*((1-$B$3)*Per_Pelanggan!$B$9+$B$3*Per_Pelanggan!$C$9)*12-Asumsi!$B$34*12</f>
-        <v>37135522.522522524</v>
+        <v>41263000.0</v>
       </c>
     </row>
     <row r="11">
@@ -2343,23 +2448,23 @@
       </c>
       <c r="B11" s="21">
         <f>$A11*B$5*((1-$B$3)*Per_Pelanggan!$B$9+$B$3*Per_Pelanggan!$C$9)*12-Asumsi!$B$34*12</f>
-        <v>14854209.00900901</v>
+        <v>16505200.000000002</v>
       </c>
       <c r="C11" s="21">
         <f>$A11*C$5*((1-$B$3)*Per_Pelanggan!$B$9+$B$3*Per_Pelanggan!$C$9)*12-Asumsi!$B$34*12</f>
-        <v>29708418.01801802</v>
+        <v>33010400.000000004</v>
       </c>
       <c r="D11" s="21">
         <f>$A11*D$5*((1-$B$3)*Per_Pelanggan!$B$9+$B$3*Per_Pelanggan!$C$9)*12-Asumsi!$B$34*12</f>
-        <v>44562627.027027026</v>
+        <v>49515600.0</v>
       </c>
       <c r="E11" s="21">
         <f>$A11*E$5*((1-$B$3)*Per_Pelanggan!$B$9+$B$3*Per_Pelanggan!$C$9)*12-Asumsi!$B$34*12</f>
-        <v>59416836.03603604</v>
+        <v>66020800.00000001</v>
       </c>
       <c r="F11" s="21">
         <f>$A11*F$5*((1-$B$3)*Per_Pelanggan!$B$9+$B$3*Per_Pelanggan!$C$9)*12-Asumsi!$B$34*12</f>
-        <v>74271045.04504505</v>
+        <v>82526000.0</v>
       </c>
     </row>
     <row r="12">
@@ -2368,23 +2473,23 @@
       </c>
       <c r="B12" s="21">
         <f>$A12*B$5*((1-$B$3)*Per_Pelanggan!$B$9+$B$3*Per_Pelanggan!$C$9)*12-Asumsi!$B$34*12</f>
-        <v>37135522.522522524</v>
+        <v>41263000.0</v>
       </c>
       <c r="C12" s="21">
         <f>$A12*C$5*((1-$B$3)*Per_Pelanggan!$B$9+$B$3*Per_Pelanggan!$C$9)*12-Asumsi!$B$34*12</f>
-        <v>74271045.04504505</v>
+        <v>82526000.0</v>
       </c>
       <c r="D12" s="21">
         <f>$A12*D$5*((1-$B$3)*Per_Pelanggan!$B$9+$B$3*Per_Pelanggan!$C$9)*12-Asumsi!$B$34*12</f>
-        <v>111406567.56756757</v>
+        <v>123789000.0</v>
       </c>
       <c r="E12" s="21">
         <f>$A12*E$5*((1-$B$3)*Per_Pelanggan!$B$9+$B$3*Per_Pelanggan!$C$9)*12-Asumsi!$B$34*12</f>
-        <v>148542090.0900901</v>
+        <v>165052000.0</v>
       </c>
       <c r="F12" s="21">
         <f>$A12*F$5*((1-$B$3)*Per_Pelanggan!$B$9+$B$3*Per_Pelanggan!$C$9)*12-Asumsi!$B$34*12</f>
-        <v>185677612.6126126</v>
+        <v>206315000.0</v>
       </c>
     </row>
     <row r="15">
@@ -2420,7 +2525,7 @@
       </c>
       <c r="B17" s="21">
         <f>(1-$B$3)*Per_Pelanggan!$B$9+$B$3*Per_Pelanggan!$C$9</f>
-        <v>6189.253753753754</v>
+        <v>6877.166666666667</v>
       </c>
     </row>
     <row r="18">
@@ -2431,7 +2536,7 @@
       </c>
       <c r="B18" s="23">
         <f>IF(B17&lt;=0,0,ROUNDUP(($B$16+Asumsi!$B$34)/B17,0))</f>
-        <v>808.0</v>
+        <v>728.0</v>
       </c>
     </row>
     <row r="19">
@@ -2452,7 +2557,7 @@
       </c>
       <c r="B20" s="23">
         <f>IF(B19&lt;=0,0,ROUNDUP(B18/B19,0))</f>
-        <v>40400.0</v>
+        <v>36400.0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>